<commit_message>
Piezo and strobe update
</commit_message>
<xml_diff>
--- a/bom/JLC_CART.xlsx
+++ b/bom/JLC_CART.xlsx
@@ -527,11 +527,11 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>0.1976</t>
+          <t>0.1064</t>
         </is>
       </c>
     </row>
@@ -562,11 +562,11 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0.1420</t>
+          <t>0.0852</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0.0643</t>
+          <t>0.0767</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -601,34 +601,34 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.9002</t>
+          <t>1.0738</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>C52306</t>
+          <t>C15850</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>CL32A226KAJNNNE</t>
+          <t>CL21A106KAYNNNE</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>22uF 25V X5R ±10% 1210 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>10uF 25V X5R ±10% 0805 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>0.1814</t>
+          <t>0.0767</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -636,34 +636,34 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>0.7256</t>
+          <t>0.3068</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>C778333</t>
+          <t>C307331</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>C0402C0G0R6B500NTB</t>
+          <t>CL05B104KB54PNC</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>0.6pF 50V C0G 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>100nF 50V X7R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>0.0029</t>
+          <t>0.0076</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -671,34 +671,34 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0.0058</t>
+          <t>0.0152</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>C3875120</t>
+          <t>C52923</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>C0402C0G500-0R8BNP</t>
+          <t>CL05A105KA5NQNC</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>0.8pF 50V C0G 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>1uF 25V X5R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>0.0105</t>
+          <t>0.0142</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.0210</t>
+          <t>0.0284</t>
         </is>
       </c>
     </row>
@@ -718,57 +718,57 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>C1547</t>
+          <t>C307331</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>0402CG120J500NT</t>
+          <t>CL05B104KB54PNC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>12pF 50V C0G ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
+          <t>100nF 50V X7R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0.0036</t>
+          <t>0.0076</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>0.0144</t>
+          <t>0.0152</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>C160352</t>
+          <t>C307331</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>B2B-PH-SM4-TB(LF)(SN)</t>
+          <t>CL05B104KB54PNC</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 100V 1x2P 2 2A 2P 2mm 6.6mm 7.95mm 7mm Auxiliary Solder Pin Beige Copper alloy PA PH Surface Mount,Vertical Tin UL94V-0 SMD,P=2mm Wire To Board Connector ROHS</t>
+          <t>100nF 50V X7R ±10% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>0.3586</t>
+          <t>0.0076</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -776,7 +776,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>0.7172</t>
+          <t>0.0152</t>
         </is>
       </c>
     </row>
@@ -788,30 +788,30 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>C2843891</t>
+          <t>C52306</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>XL-3030UWC-1W-3V</t>
+          <t>CL32A226KAJNNNE</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 120° 1W 3.4V 350mA 6500K~7000K Discrete Diode Top-mount White Yellow Lens SMD3030-2P LED Indication - Discrete ROHS</t>
+          <t>22uF 25V X5R ±10% 1210 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>0.042</t>
+          <t>0.1812</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>0.672</t>
+          <t>0.7248</t>
         </is>
       </c>
     </row>
@@ -823,22 +823,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>C151304</t>
+          <t>C778333</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>SP3012-04UTG</t>
+          <t>C0402C0G0R6B500NTB</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+125℃ 0.5pF 1.5uA 4A@8/20us 5V 8.4V ESD Four channels IEC 61000-4-2、IEC 61000-4-5、IEC 61000-4-4 UDFN-10(1x2.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
+          <t>0.6pF 50V C0G 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>0.2974</t>
+          <t>0.0029</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>0.5948</t>
+          <t>0.0058</t>
         </is>
       </c>
     </row>
@@ -858,22 +858,22 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>C2827688</t>
+          <t>C3875120</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>PRTR5V0U2X</t>
+          <t>C0402C0G500-0R8BNP</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 0.3pF、0.8pF 100W 10V、15V 5V 6.5V 6A 80nA ESD IEC 61000-4-2、IEC 61000-4-5、IEC 61000-4-4 Three channels Unidirectional SOT-143 ESD and Surge Protection (TVS/ESD) ROHS</t>
+          <t>0.8pF 50V C0G 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>0.0609</t>
+          <t>0.0105</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -881,7 +881,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>0.1218</t>
+          <t>0.0210</t>
         </is>
       </c>
     </row>
@@ -893,30 +893,30 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>C8678</t>
+          <t>C1547</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>SS34</t>
+          <t>0402CG120J500NT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 3A 40V 500uA@40V 550mV@3A Independent SMA(DO-214AC) Schottky Diodes ROHS</t>
+          <t>12pF 50V C0G ±5% 0402 Multilayer Ceramic Capacitors MLCC - SMD/SMT ROHS</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>0.0301</t>
+          <t>0.0036</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>0.1806</t>
+          <t>0.0144</t>
         </is>
       </c>
     </row>
@@ -928,22 +928,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>C146125</t>
+          <t>C131339</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>XH-2PVertical welding</t>
+          <t>B3B-PH-K-S(LF)(SN)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 12mm 1x2P 2 2.5mm 250V 2P 3A 6mm 7.8mm Beige LCP Phosphor bronze Surface Mount,Vertical Tin UL94V-0 XH SMD,P=2.5mm Wire To Board Connector ROHS</t>
+          <t>-25℃~+85℃ 1 100V 1x3P 2A 2mm 3 3P 4.5mm 6mm 7.9mm Brass K Pin PA66 PH Through Hole Tin UL94V-0 White 插件,P=2mm Wire To Board Connector ROHS</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>0.0669</t>
+          <t>0.0412</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -951,7 +951,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>0.1338</t>
+          <t>0.0824</t>
         </is>
       </c>
     </row>
@@ -963,30 +963,30 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>C2681544</t>
+          <t>C2843891</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2.54-3P LT</t>
+          <t>XL-3030UWC-1W-3V</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 1x3P 2.5mm 250V 3 3A 3P Beige Brass LCP Surface Mount,Vertical Tin UL94V-0 XH SMD,P=2.5mm Wire To Board Connector ROHS</t>
+          <t>-40℃~+85℃ 120° 1W 3.4V 350mA 6500K~7000K Discrete Diode Top-mount White Yellow Lens SMD3030-2P LED Indication - Discrete ROHS</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>0.0814</t>
+          <t>0.042</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>0.1628</t>
+          <t>0.672</t>
         </is>
       </c>
     </row>
@@ -998,22 +998,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>C266888</t>
+          <t>C151304</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>SMN-303</t>
+          <t>SP3012-04UTG</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1.37mm Connector and Ejector Nano-SIM Card Push-Push With Card Detect SMD SIM Card Connectors ROHS</t>
+          <t>-40℃~+125℃ 0.5pF 1.5uA 4A@8/20us 5V 8.4V ESD Four channels IEC 61000-4-2、IEC 61000-4-5、IEC 61000-4-4 UDFN-10(1x2.5) ESD and Surge Protection (TVS/ESD) ROHS</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>0.4894</t>
+          <t>0.297</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>0.9788</t>
+          <t>0.594</t>
         </is>
       </c>
     </row>
@@ -1033,65 +1033,65 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>C2849472</t>
+          <t>C2827688</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>PNLS4030-100M 10UH</t>
+          <t>PRTR5V0U2X</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>10uH 120mΩ 2A 2A Magnetic Shielded Inductor ±20% SMD,4x4mm Power Inductors ROHS</t>
+          <t>-55℃~+125℃ 0.3pF、0.8pF 100W 10V、15V 5V 6.5V 6A 80nA ESD IEC 61000-4-2、IEC 61000-4-5、IEC 61000-4-4 Three channels Unidirectional SOT-143 ESD and Surge Protection (TVS/ESD) ROHS</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>0.0521</t>
+          <t>0.0609</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>0.2084</t>
+          <t>0.1218</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>C92959</t>
+          <t>C8678</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>NRS4018T2R2MDGJ</t>
+          <t>SS34</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2.2A 2.2uH 3A 42mΩ ±20% SMD,4x4mm Power Inductors ROHS</t>
+          <t>-55℃~+125℃ 3A 40V 500uA@40V 550mV@3A Independent SMA(DO-214AC) Schottky Diodes ROHS</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>0.0886</t>
+          <t>0.0301</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>0.3544</t>
+          <t>0.1806</t>
         </is>
       </c>
     </row>
@@ -1103,22 +1103,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>C86065</t>
+          <t>C146125</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>LQG15HS4N7S02D</t>
+          <t>XH-2PVertical welding</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>160mΩ 4.7nH 6GHz 700mA 8@100MHz Multilayer inductor 0402 Inductors (SMD) ROHS</t>
+          <t>-25℃~+85℃ 1 12mm 1x2P 2 2.5mm 250V 2P 3A 6mm 7.8mm Beige LCP Phosphor bronze Surface Mount,Vertical Tin UL94V-0 XH SMD,P=2.5mm Wire To Board Connector ROHS</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>0.023</t>
+          <t>0.0668</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>0.046</t>
+          <t>0.1336</t>
         </is>
       </c>
     </row>
@@ -1138,30 +1138,30 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>C60105</t>
+          <t>C2681544</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>19-237/R6GHBHC-A01/2T</t>
+          <t>2.54-3P LT</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>120° Common Anode SMD-4P,1.6x1.6mm RGB LEDs ROHS</t>
+          <t>-25℃~+85℃ 1 1x3P 2.5mm 250V 3 3A 3P Beige Brass LCP Surface Mount,Vertical Tin UL94V-0 XH SMD,P=2.5mm Wire To Board Connector ROHS</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>0.0624</t>
+          <t>0.0814</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>0.2496</t>
+          <t>0.1628</t>
         </is>
       </c>
     </row>
@@ -1173,22 +1173,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>C456012</t>
+          <t>C266888</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>TYPE-C 6P</t>
+          <t>SMN-303</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 3,000 Cycles 3A 5V 6P Black Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
+          <t>-25℃~+85℃ 1.37mm Connector and Ejector Nano-SIM Card Push-Push With Card Detect SMD SIM Card Connectors ROHS</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>0.0385</t>
+          <t>0.4888</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>0.0770</t>
+          <t>0.9776</t>
         </is>
       </c>
     </row>
@@ -1208,92 +1208,92 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>C3018484</t>
+          <t>C2849472</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>BSS84</t>
+          <t>PNLS4030-100M 10UH</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+150℃ 1 P-Channel 10pF 10Ω@5V 130mA 225mW 2V 30pF 50V 5pF SOT-23 MOSFETs ROHS</t>
+          <t>10uH 120mΩ 2A 2A Magnetic Shielded Inductor ±20% SMD,4x4mm Power Inductors ROHS</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>0.0223</t>
+          <t>0.052</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>0.1338</t>
+          <t>0.208</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>C8545</t>
+          <t>C92959</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>2N7002</t>
+          <t>NRS4018T2R2MDGJ</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1 N-channel 115mA 2.5V 225mW 50pF 5pF 5Ω@10V 60V SOT-23 MOSFETs ROHS</t>
+          <t>2.2A 2.2uH 3A 42mΩ ±20% SMD,4x4mm Power Inductors ROHS</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>0.0154</t>
+          <t>0.0884</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>0.0924</t>
+          <t>0.3536</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>C25792</t>
+          <t>C86065</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>0402WGF4702TCE</t>
+          <t>LQG15HS4N7S02D</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>160mΩ 4.7nH 6GHz 700mA 8@100MHz Multilayer inductor 0402 Inductors (SMD) ROHS</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>0.0012</t>
+          <t>0.023</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>0.0024</t>
+          <t>0.046</t>
         </is>
       </c>
     </row>
@@ -1313,65 +1313,65 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>C22369540</t>
+          <t>C60105</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>RCA02150KFLF</t>
+          <t>19-237/R6GHBHC-A01/2T</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 150kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>120° Common Anode SMD-4P,1.6x1.6mm RGB LEDs ROHS</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>0.0004</t>
+          <t>0.0623</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.2492</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>C49330233</t>
+          <t>C8545</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>AS0210KF</t>
+          <t>2N7002</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 10kΩ 50V 62.5mW ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>1 N-channel 115mA 2.5V 225mW 50pF 5pF 5Ω@10V 60V SOT-23 MOSFETs ROHS</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.0153</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>0.0128</t>
+          <t>0.0306</t>
         </is>
       </c>
     </row>
@@ -1383,17 +1383,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>C25104</t>
+          <t>C25792</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>0402WGF3300TCE</t>
+          <t>0402WGF4702TCE</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 330Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 47kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1402,11 +1402,11 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>0.0072</t>
+          <t>0.0024</t>
         </is>
       </c>
     </row>
@@ -1418,162 +1418,162 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>C25169</t>
+          <t>C22369540</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>0402WGJ047JTCE</t>
+          <t>RCA02150KFLF</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7Ω 50V 62.5mW Thick Film Resistor ±200ppm/℃ ±5% 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 150kΩ 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>0.0256</t>
+          <t>0.0008</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>C25905</t>
+          <t>C49330233</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>0402WGF5101TCE</t>
+          <t>AS0210KF</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 5.1kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 10kΩ 50V 62.5mW ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>0.0009</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.0128</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>C100318</t>
+          <t>C25104</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CR0402FF22R0G</t>
+          <t>0402WGF3300TCE</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+125℃ 22Ω 50V 62.5mW Thick Film Resistor ±1% ±200ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 330Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>0.0024</t>
+          <t>0.0072</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>C25076</t>
+          <t>C175252</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>0402WGF1000TCE</t>
+          <t>CRH2512F22R0E04Z</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 200V 22Ω 2W Thick Film Resistor ±1% ±100ppm/℃ 2512 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>0.0012</t>
+          <t>0.0589</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>0.0072</t>
+          <t>0.4712</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>C159084</t>
+          <t>C25076</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>RTT021913FTH</t>
+          <t>0402WGF1000TCE</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 191kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100Ω 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>0.0007</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>0.0024</t>
         </is>
       </c>
     </row>
@@ -1593,22 +1593,22 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>C64043</t>
+          <t>C159084</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>0402WGF2403TCE</t>
+          <t>RTT021913FTH</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 240kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 191kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.0007</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.0014</t>
         </is>
       </c>
     </row>
@@ -1628,22 +1628,22 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>C144809</t>
+          <t>C64043</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>AC0402FR-07100KL</t>
+          <t>0402WGF2403TCE</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 240kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>0.0018</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -1651,77 +1651,77 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>0.0036</t>
+          <t>0.002</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Basic</t>
+          <t>Extended</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>C25900</t>
+          <t>C144809</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>0402WGF4701TCE</t>
+          <t>AC0402FR-07100KL</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
+          <t>-55℃~+155℃ 100kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>0.0011</t>
+          <t>0.0018</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>0.0044</t>
+          <t>0.0036</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Extended</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>C719176</t>
+          <t>C25900</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>TC33X-2-103E</t>
+          <t>0402WGF4701TCE</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>1 10kΩ 150mW ±25% ±250ppm/℃ SMD-3P,3.8x3.6mm Potentiometers, Variable Resistors ROHS</t>
+          <t>-55℃~+155℃ 4.7kΩ 50V 62.5mW Thick Film Resistor ±1% ±100ppm/℃ 0402 Chip Resistor - Surface Mount ROHS</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>0.1065</t>
+          <t>0.0011</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>0.2130</t>
+          <t>0.0044</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>0.0629</t>
+          <t>0.0628</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>0.1258</t>
+          <t>0.1256</t>
         </is>
       </c>
     </row>
@@ -1768,22 +1768,22 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>C77131</t>
+          <t>C190794</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>NCP15XH103F03RC</t>
+          <t>NRF52840-QIAA-R</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+125℃ 0.5mm 100mW 10kΩ 1mW/℃ 1mm 310uA 3380K 3434K 3455K ±1% ±1% 0402 NTC Thermistors ROHS</t>
+          <t>-95dBm 1.7V~5.5V 2.4GHz 2.4GHz~2.4835GHz 2Mbps 4.82mA 6.26mA 8dBm SPI、USB、UART、ADC、I2S、PWM ZigBee、Bluetooth、LoRa、ISM transceiver AQFN-73-EP(7x7) RF Transceiver ICs ROHS</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>0.0199</t>
+          <t>5.7315</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>0.0398</t>
+          <t>11.4630</t>
         </is>
       </c>
     </row>
@@ -1803,22 +1803,22 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>C190794</t>
+          <t>C22397843</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>NRF52840-QIAA-R</t>
+          <t>nRF9151-LACA-R7</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>-95dBm 1.7V~5.5V 2.4GHz 2.4GHz~2.4835GHz 2Mbps 4.82mA 6.26mA 8dBm SPI、USB、UART、ADC、I2S、PWM ZigBee、Bluetooth、LoRa、ISM transceiver AQFN-73-EP(7x7) RF Transceiver ICs ROHS</t>
+          <t>LGA-113(12.1x11.1) RF Modules ROHS</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>5.7384</t>
+          <t>16.1232</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>11.4768</t>
+          <t>32.2464</t>
         </is>
       </c>
     </row>
@@ -1838,22 +1838,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>C22397843</t>
+          <t>C25346894</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>nRF9151-LACA-R7</t>
+          <t>NPM1300-CAAA-R7</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>LGA-113(12.1x11.1) RF Modules ROHS</t>
+          <t>WLCSP-35(2.4x3.1) Power Management - Specialized ROHS</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>16.1428</t>
+          <t>2.6665</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>32.2856</t>
+          <t>5.3330</t>
         </is>
       </c>
     </row>
@@ -1873,22 +1873,22 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>C25346894</t>
+          <t>C437655</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>NPM1300-CAAA-R7</t>
+          <t>BMA400</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>WLCSP-35(2.4x3.1) Power Management - Specialized ROHS</t>
+          <t>-40℃~+85℃ 1.71V~3.6V 12bit 160nA 1KB Accelerometer SPI、I2C X,Y,Z ±16g LGA-12(2x2) Accelerometers ROHS</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2.5632</t>
+          <t>2.3923</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>5.1264</t>
+          <t>4.7846</t>
         </is>
       </c>
     </row>
@@ -1908,30 +1908,30 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>C437655</t>
+          <t>C5137195</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>BMA400</t>
+          <t>BWU.FL-IPEX1</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1.71V~3.6V 12bit 160nA 1KB Accelerometer SPI、I2C X,Y,Z ±16g LGA-12(2x2) Accelerometers ROHS</t>
+          <t>1 1.25mm 2mm 50Ω 6GHz Board Side IPEX Male Pin SMD Coaxial Connectors (RF) ROHS</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2.3952</t>
+          <t>0.0397</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>4.7904</t>
+          <t>0.1588</t>
         </is>
       </c>
     </row>
@@ -1943,30 +1943,30 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>C5137195</t>
+          <t>C239238</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>BWU.FL-IPEX1</t>
+          <t>AN6520-245</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>1 1.25mm 2mm 50Ω 6GHz Board Side IPEX Male Pin SMD Coaxial Connectors (RF) ROHS</t>
+          <t>-40℃~+85℃ 0.5dBi 1mm 2 2.2mm 2.45GHz 200MHz 3W 50Ω 6.5mm SMD Antennas ROHS</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>0.0398</t>
+          <t>0.5727</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>0.1592</t>
+          <t>1.1454</t>
         </is>
       </c>
     </row>
@@ -1978,22 +1978,22 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>C239238</t>
+          <t>C160405</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>AN6520-245</t>
+          <t>SM06B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 0.5dBi 1mm 2 2.2mm 2.45GHz 200MHz 3W 50Ω 6.5mm SMD Antennas ROHS</t>
+          <t>-25℃~+85℃ 1 1A 1mm 1x6P 2.9mm 4.32mm 50V 6 6P 8mm Auxiliary Solder Pin Copper alloy PA SH Surface Mount, Right Angle Tin UL94V-0 White SMD,P=1mm,卧贴 Wire To Board Connector ROHS</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>0.5734</t>
+          <t>0.2994</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>1.1468</t>
+          <t>0.5988</t>
         </is>
       </c>
     </row>
@@ -2013,22 +2013,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>C160405</t>
+          <t>C160404</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>SM06B-SRSS-TB(LF)(SN)</t>
+          <t>SM04B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 1A 1mm 1x6P 2.9mm 4.32mm 50V 6 6P 8mm Auxiliary Solder Pin Copper alloy PA SH Surface Mount, Right Angle Tin UL94V-0 White SMD,P=1mm,卧贴 Wire To Board Connector ROHS</t>
+          <t>-25℃~+85℃ 1 1A 1mm 1x4P 2.9mm 4 4.32mm 4P 50V 6mm Auxiliary Solder Pin Copper alloy PA SH Surface Mount, Right Angle Tin UL94V-0 White SMD,P=1mm,卧贴 Wire To Board Connector ROHS</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>0.2998</t>
+          <t>0.2243</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>0.5996</t>
+          <t>0.4486</t>
         </is>
       </c>
     </row>
@@ -2048,30 +2048,30 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>C160404</t>
+          <t>C41376037</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB(LF)(SN)</t>
+          <t>HX PZ1.27-2x5P TP</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>-25℃~+85℃ 1 1A 1mm 1x4P 2.9mm 4 4.32mm 4P 50V 6mm Auxiliary Solder Pin Copper alloy PA SH Surface Mount, Right Angle Tin UL94V-0 White SMD,P=1mm,卧贴 Wire To Board Connector ROHS</t>
+          <t>-40℃~+105℃ 1.27mm 1.27mm 10P 1A 1mm 2 2x5P 4mm 500V Black Brass Gold Pin Header Surface Mount,Vertical SMD,P=1.27mm Pin Headers ROHS</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>0.2245</t>
+          <t>0.0959</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>0.4490</t>
+          <t>0.3836</t>
         </is>
       </c>
     </row>
@@ -2083,22 +2083,22 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>C41376037</t>
+          <t>C84817</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>HX PZ1.27-2x5P TP</t>
+          <t>MT3608</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+105℃ 1.27mm 1.27mm 10P 1A 1mm 2 2x5P 4mm 500V Black Brass Gold Pin Header Surface Mount,Vertical SMD,P=1.27mm Pin Headers ROHS</t>
+          <t>-40℃~+85℃ 1 1.2MHz 100uA、1.6mA 2A 2V~24V Adjustable Boost Boost Built-in No SOT-23-6 DC-DC Converters ROHS</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>0.096</t>
+          <t>0.0799</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>0.384</t>
+          <t>0.3196</t>
         </is>
       </c>
     </row>
@@ -2118,30 +2118,30 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>C84817</t>
+          <t>C2765186</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>MT3608</t>
+          <t>TYPE-C 16PIN 2MD(073)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>-40℃~+85℃ 1 1.2MHz 100uA、1.6mA 2A 2V~24V Adjustable Boost Boost Built-in No SOT-23-6 DC-DC Converters ROHS</t>
+          <t>-25℃~+85℃ 1 16P 3A 5,000 times 5V Black Female Surface Mount, Right Angle Type-C SMD USB Connectors ROHS</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.0736</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>0.32</t>
+          <t>0.1472</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>0.2321</t>
+          <t>0.2319</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>0.4642</t>
+          <t>0.4638</t>
         </is>
       </c>
     </row>

</xml_diff>